<commit_message>
feat: exportacao em PDF (jsPDF), linha de Total nas exportacoes, e renomear categoria Pediatricas/congenitas para Congenitas
</commit_message>
<xml_diff>
--- a/data/procedimentos.xlsx
+++ b/data/procedimentos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Procedimentos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Como usar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Procedimentos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Como usar" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -489,7 +489,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -526,7 +526,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -600,7 +600,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -748,7 +748,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -896,7 +896,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -933,7 +933,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1303,7 +1303,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1451,7 +1451,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1636,7 +1636,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1673,7 +1673,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1821,7 +1821,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2080,7 +2080,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2117,7 +2117,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2635,7 +2635,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2746,7 +2746,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -2820,7 +2820,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -2894,7 +2894,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -2968,7 +2968,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3005,7 +3005,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3042,7 +3042,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3116,7 +3116,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3153,7 +3153,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3227,7 +3227,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3301,7 +3301,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3338,7 +3338,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3375,7 +3375,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3412,7 +3412,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3449,7 +3449,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -3486,7 +3486,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3523,7 +3523,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Pediátricas/congênitas</t>
+          <t>Congênitas</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">

</xml_diff>